<commit_message>
Skizzen-Vorschlag nur aus Grundformen (wep-skizze/2), Bausteine, Linienstärke
- Vorschlag kennt keine fertigen Symbole mehr: Rechteck, Ellipse, Vieleck (Dreieck, offener Linienzug), Bogen, Linie, Maßlinie, Text
- Jede Form gefüllt, eigene Linienfarbe, -stärke (pt) und -art; name, bezug; frei gezeichnete Reihenfolge im Excel
- window.wep.skizze.baustein(): fertige Grundformen (Baum, Hecke, Tor, Kompost, Entfernen …) nach dem Skill parzellen-skizze
- Editor, PNG/PDF, Excel-Export: Linienstärke, offene Linienzüge, Textfarbe/-größe, Namen
- Fix: Treffertest offener Linienzüge
- Doku, Tests, Durchlauf mit Screenshots

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4ZanQZQtLWDxL4PGpWa8v
</commit_message>
<xml_diff>
--- a/docs/skizze-agent/export.xlsx
+++ b/docs/skizze-agent/export.xlsx
@@ -18056,6 +18056,211 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>97157</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>70014</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>15237</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>110012</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="25" name="L" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1925957" y="4337214"/>
+          <a:ext cx="1775455" cy="1182998"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E7E6E6"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="262626"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-DE" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t>L</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>15237</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>175263</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>607693</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>110012</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="26" name="A1" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="3701412" y="4632963"/>
+          <a:ext cx="592456" cy="887249"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="E7E6E6"/>
+        </a:solidFill>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="262626"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-DE" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t>A1</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>97157</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>24761</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>985363</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>45718</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="27" name="K" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1925957" y="5815961"/>
+          <a:ext cx="888206" cy="592457"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="19050">
+          <a:solidFill>
+            <a:srgbClr val="262626"/>
+          </a:solidFill>
+          <a:prstDash val="dash"/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-DE" sz="1100">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t>K</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>547059</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>127009</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>902659</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>101609</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="28" name="Flieder_0" descr="wep-app"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
+          <a:extLst>
+            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
+              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1156659" y="2679709"/>
+          <a:ext cx="355600" cy="355600"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>133359</xdr:colOff>
       <xdr:row>8</xdr:row>
@@ -18069,7 +18274,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="Vieleck_0" descr="wep-app"/>
+        <xdr:cNvPr id="29" name="Wiese_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -18132,6 +18337,62 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
+      <xdr:colOff>689613</xdr:colOff>
+      <xdr:row>11</xdr:row>
+      <xdr:rowOff>94310</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1725215</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>29059</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="30" name="Dreieckbeet_0" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="2518413" y="2266010"/>
+          <a:ext cx="1035602" cy="887249"/>
+        </a:xfrm>
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="1035602" h="887249">
+              <a:moveTo>
+                <a:pt x="0" y="0"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="1035602" y="0"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="0" y="887249"/>
+              </a:lnTo>
+              <a:close/>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="EBDDC7"/>
+        </a:solidFill>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:srgbClr val="7030A0"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>3</xdr:col>
       <xdr:colOff>1074375</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>44760</xdr:rowOff>
@@ -18144,7 +18405,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="26" name="Weg_0" descr="wep-app"/>
+        <xdr:cNvPr id="31" name="Weg_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -18186,416 +18447,115 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1310783</xdr:colOff>
+      <xdr:colOff>1695545</xdr:colOff>
       <xdr:row>45</xdr:row>
       <xdr:rowOff>7988</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1665874</xdr:colOff>
+      <xdr:colOff>1695545</xdr:colOff>
       <xdr:row>46</xdr:row>
       <xdr:rowOff>172579</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="27" name="Tor_0" descr="wep-app"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId4"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="32" name="Tor_0" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3139583" y="8656688"/>
-          <a:ext cx="355091" cy="355091"/>
+          <a:off x="3524345" y="8656688"/>
+          <a:ext cx="0" cy="355091"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:srgbClr val="262626"/>
+          </a:solidFill>
+        </a:ln>
       </xdr:spPr>
-    </xdr:pic>
+    </xdr:cxnSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>97157</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>70014</xdr:rowOff>
+      <xdr:colOff>1340454</xdr:colOff>
+      <xdr:row>45</xdr:row>
+      <xdr:rowOff>7988</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>15237</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>110012</xdr:rowOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>1695545</xdr:colOff>
+      <xdr:row>46</xdr:row>
+      <xdr:rowOff>172579</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="L" descr="wep-app"/>
+        <xdr:cNvPr id="33" name="Tor_Bogen_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1925957" y="4337214"/>
-          <a:ext cx="1775455" cy="1182998"/>
+          <a:off x="3169254" y="8656688"/>
+          <a:ext cx="355091" cy="355091"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
+        <a:custGeom>
           <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="E7E6E6"/>
-        </a:solidFill>
-        <a:ln w="19050">
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="355091" h="355091">
+              <a:moveTo>
+                <a:pt x="0" y="355091"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="2871" y="309149"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="11485" y="263208"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="26799" y="219180"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="47856" y="177067"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="72741" y="138782"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="103369" y="104326"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="138782" y="73698"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="177067" y="47856"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="219180" y="26799"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="263207" y="12443"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="308192" y="2872"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="355091" y="0"/>
+              </a:lnTo>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:noFill/>
+        <a:ln w="12700">
           <a:solidFill>
             <a:srgbClr val="262626"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:rPr>
-            <a:t>L</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>15237</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>175263</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>607693</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>110012</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="29" name="A1" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3701412" y="4632963"/>
-          <a:ext cx="592456" cy="887249"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="E7E6E6"/>
-        </a:solidFill>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:srgbClr val="262626"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:rPr>
-            <a:t>A1</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>97157</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>24761</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>985363</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>45718</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="30" name="K" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1925957" y="5815961"/>
-          <a:ext cx="888206" cy="592457"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln w="19050">
-          <a:solidFill>
-            <a:srgbClr val="262626"/>
-          </a:solidFill>
-          <a:prstDash val="dash"/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="de-DE" sz="1100">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:rPr>
-            <a:t>K</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>547059</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>127009</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>902659</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>101609</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="31" name="Flieder_0" descr="wep-app"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId5">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId6"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1156659" y="2679709"/>
-          <a:ext cx="355600" cy="355600"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>677562</xdr:colOff>
-      <xdr:row>13</xdr:row>
-      <xdr:rowOff>25331</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>206354</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>12788</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="32" name="Apfel_0" descr="wep-app"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId7">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId8"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4363737" y="2578031"/>
-          <a:ext cx="452717" cy="558957"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>345136</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>1034</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>150153</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>178991</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="33" name="Apfel_1" descr="wep-app"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId10"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4955236" y="4649234"/>
-          <a:ext cx="452717" cy="558957"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>49387</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>61989</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>502104</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>49446</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="34" name="Birne_0" descr="wep-app"/>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId11">
-          <a:extLst>
-            <a:ext uri="{96DAC541-7B7A-43D3-8B79-37D633B846F1}">
-              <asvg:svgBlip xmlns:asvg="http://schemas.microsoft.com/office/drawing/2016/SVG/main" r:embed="rId12"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4659487" y="6424689"/>
-          <a:ext cx="452717" cy="558957"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>18</xdr:row>
-      <xdr:rowOff>92162</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>167741</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="35" name="Liguster-Hecke_0_0" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5371239" y="3597362"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
@@ -18604,36 +18564,36 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>19</xdr:row>
-      <xdr:rowOff>86018</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>868986</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>170779</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>161597</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>13016</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>181274</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="36" name="Liguster-Hecke_0_1" descr="wep-app"/>
+        <xdr:cNvPr id="34" name="baum_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5435097" y="3781718"/>
-          <a:ext cx="266079" cy="266079"/>
+          <a:off x="4555161" y="2913979"/>
+          <a:ext cx="67955" cy="200995"/>
         </a:xfrm>
-        <a:prstGeom prst="ellipse">
+        <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
+          <a:srgbClr val="7F5A2E"/>
         </a:solidFill>
         <a:ln w="12700">
           <a:solidFill>
-            <a:srgbClr val="548235"/>
+            <a:srgbClr val="7F5A2E"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
@@ -18642,36 +18602,36 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>79873</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>690962</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>181341</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>155452</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>914928</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>24307</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="37" name="Liguster-Hecke_0_2" descr="wep-app"/>
+        <xdr:cNvPr id="35" name="baum_1" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5371239" y="3966073"/>
-          <a:ext cx="266079" cy="266079"/>
+          <a:off x="4377137" y="2734041"/>
+          <a:ext cx="223966" cy="223966"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
+          <a:srgbClr val="548235"/>
         </a:solidFill>
         <a:ln w="12700">
           <a:solidFill>
-            <a:srgbClr val="548235"/>
+            <a:srgbClr val="385723"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
@@ -18680,36 +18640,36 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>73729</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>891957</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>181341</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>149308</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>191998</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>24307</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="38" name="Liguster-Hecke_0_3" descr="wep-app"/>
+        <xdr:cNvPr id="36" name="baum_2" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5435097" y="4150429"/>
-          <a:ext cx="266079" cy="266079"/>
+          <a:off x="4578132" y="2734041"/>
+          <a:ext cx="223966" cy="223966"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
+          <a:srgbClr val="548235"/>
         </a:solidFill>
         <a:ln w="12700">
           <a:solidFill>
-            <a:srgbClr val="548235"/>
+            <a:srgbClr val="385723"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
@@ -18718,36 +18678,36 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>67585</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>758917</xdr:colOff>
+      <xdr:row>13</xdr:row>
+      <xdr:rowOff>35859</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>143164</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>124042</xdr:colOff>
+      <xdr:row>14</xdr:row>
+      <xdr:rowOff>134409</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="39" name="Liguster-Hecke_0_4" descr="wep-app"/>
+        <xdr:cNvPr id="37" name="baum_3" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5371239" y="4334785"/>
-          <a:ext cx="266079" cy="266079"/>
+          <a:off x="4445092" y="2588559"/>
+          <a:ext cx="289050" cy="289050"/>
         </a:xfrm>
         <a:prstGeom prst="ellipse">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
+          <a:srgbClr val="548235"/>
         </a:solidFill>
         <a:ln w="12700">
           <a:solidFill>
-            <a:srgbClr val="548235"/>
+            <a:srgbClr val="385723"/>
           </a:solidFill>
         </a:ln>
       </xdr:spPr>
@@ -18756,721 +18716,25 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>61440</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>746475</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>26187</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>137019</xdr:rowOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>238475</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>26187</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="40" name="Liguster-Hecke_0_5" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5435097" y="4519140"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>55296</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>130875</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="41" name="Liguster-Hecke_0_6" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5371239" y="4703496"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>25</xdr:row>
-      <xdr:rowOff>49152</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>124731</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="42" name="Liguster-Hecke_0_7" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5435097" y="4887852"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>43008</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>118587</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="43" name="Liguster-Hecke_0_8" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5371239" y="5072208"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>36863</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>112442</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="44" name="Liguster-Hecke_0_9" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5435097" y="5256563"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>30719</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>106298</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="45" name="Liguster-Hecke_0_10" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5371239" y="5440919"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>29</xdr:row>
-      <xdr:rowOff>24575</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>100154</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="46" name="Liguster-Hecke_0_11" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5435097" y="5625275"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>113439</xdr:colOff>
-      <xdr:row>30</xdr:row>
-      <xdr:rowOff>18430</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>379518</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>94009</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="47" name="Liguster-Hecke_0_12" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5371239" y="5809630"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>177297</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>12286</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>443376</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>87865</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="48" name="Liguster-Hecke_0_13" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5435097" y="5993986"/>
-          <a:ext cx="266079" cy="266079"/>
-        </a:xfrm>
-        <a:prstGeom prst="ellipse">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="A9D18E"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>192701</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>42612</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>666474</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>147862</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="49" name="Kompost_0" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="802301" y="7738812"/>
-          <a:ext cx="473773" cy="295750"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="D9C3A5"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="8B5A2B"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>295269</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>55312</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>327019</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>135162</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="50" name="Kompost_0_Latte_0" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="904869" y="7751512"/>
-          <a:ext cx="31750" cy="270350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="8B5A2B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>413713</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>55312</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>445463</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>135162</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="51" name="Kompost_0_Latte_1" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1023313" y="7751512"/>
-          <a:ext cx="31750" cy="270350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="8B5A2B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>532156</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>55312</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>563906</xdr:colOff>
-      <xdr:row>41</xdr:row>
-      <xdr:rowOff>135162</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="52" name="Kompost_0_Latte_2" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1141756" y="7751512"/>
-          <a:ext cx="31750" cy="270350"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="8B5A2B"/>
-        </a:solidFill>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>524821</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>80475</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>923939</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>98593</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="53" name="Blaufichte_entfernen_0" descr="wep-app"/>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1134421" y="4728675"/>
-          <a:ext cx="399118" cy="399118"/>
-        </a:xfrm>
-        <a:prstGeom prst="star16">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:srgbClr val="70AD47"/>
-        </a:solidFill>
-        <a:ln w="12700">
-          <a:solidFill>
-            <a:srgbClr val="548235"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>604645</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>160299</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>844116</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>18770</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="54" name="Blaufichte_entfernen_0_X1" descr="wep-app"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="1214245" y="4808499"/>
-          <a:ext cx="239471" cy="239471"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="25400">
-          <a:solidFill>
-            <a:srgbClr val="C00000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>604645</xdr:colOff>
-      <xdr:row>24</xdr:row>
-      <xdr:rowOff>160299</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>844116</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>18770</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="55" name="Blaufichte_entfernen_0_X2" descr="wep-app"/>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm flipH="1">
-          <a:off x="1214245" y="4808499"/>
-          <a:ext cx="239471" cy="239471"/>
-        </a:xfrm>
-        <a:prstGeom prst="straightConnector1">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="25400">
-          <a:solidFill>
-            <a:srgbClr val="C00000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>454032</xdr:colOff>
-      <xdr:row>15</xdr:row>
-      <xdr:rowOff>114309</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>995687</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>114309</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="56" name="Flieder_0_Text" descr="wep-app"/>
+        <xdr:cNvPr id="38" name="baum_4" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1063632" y="3048009"/>
-          <a:ext cx="541655" cy="190500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="de-DE" sz="900">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:rPr>
-            <a:t>Flieder</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>695958</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>25488</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>187958</xdr:colOff>
-      <xdr:row>17</xdr:row>
-      <xdr:rowOff>25488</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="57" name="Apfel_0_Text" descr="wep-app"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4382133" y="3149688"/>
-          <a:ext cx="415925" cy="190500"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="de-DE" sz="900">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-            </a:rPr>
-            <a:t>Apfel</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>4</xdr:col>
-      <xdr:colOff>846132</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>1191</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>338132</xdr:colOff>
-      <xdr:row>28</xdr:row>
-      <xdr:rowOff>1191</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="58" name="Apfel_1_Text" descr="wep-app"/>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4532307" y="5220891"/>
+          <a:off x="4432650" y="3150387"/>
           <a:ext cx="415925" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -19503,24 +18767,378 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>67783</xdr:colOff>
-      <xdr:row>36</xdr:row>
-      <xdr:rowOff>62146</xdr:rowOff>
+      <xdr:colOff>300152</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>41233</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>483708</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>62146</xdr:rowOff>
+      <xdr:colOff>368107</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>51728</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="59" name="Birne_0_Text" descr="wep-app"/>
+        <xdr:cNvPr id="39" name="baum_5" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4910252" y="4689433"/>
+          <a:ext cx="67955" cy="200995"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="7F5A2E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="7F5A2E"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>122128</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>50838</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>346094</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>84304</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="40" name="baum_6" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4732228" y="4508538"/>
+          <a:ext cx="223966" cy="223966"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>323123</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>50838</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>547089</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>84304</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="41" name="baum_7" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4933223" y="4508538"/>
+          <a:ext cx="223966" cy="223966"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>190083</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>96813</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>479133</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>4863</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="42" name="baum_8" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4800183" y="4364013"/>
+          <a:ext cx="289050" cy="289050"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>177641</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>87142</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>593566</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>87142</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="43" name="baum_9" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4677883" y="6996346"/>
+          <a:off x="4787741" y="4925842"/>
+          <a:ext cx="415925" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-DE" sz="900">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t>Apfel</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>240810</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>16937</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>308765</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>27432</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="44" name="baum_10" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4850910" y="6760637"/>
+          <a:ext cx="67955" cy="200995"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="7F5A2E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="7F5A2E"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>62786</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>26542</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>286752</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>60008</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="45" name="baum_11" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4672886" y="6579742"/>
+          <a:ext cx="223966" cy="223966"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>263781</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>26542</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>487747</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>60008</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="46" name="baum_12" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4873881" y="6579742"/>
+          <a:ext cx="223966" cy="223966"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>130742</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>72517</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>419792</xdr:colOff>
+      <xdr:row>34</xdr:row>
+      <xdr:rowOff>171067</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="47" name="baum_13" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4740842" y="6435217"/>
+          <a:ext cx="289050" cy="289050"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="548235"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="385723"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>118299</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>62845</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>534224</xdr:colOff>
+      <xdr:row>37</xdr:row>
+      <xdr:rowOff>62845</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="48" name="baum_14" descr="wep-app"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="4728399" y="6997045"/>
           <a:ext cx="415925" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -19552,26 +19170,558 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>7</xdr:col>
-      <xdr:colOff>13613</xdr:colOff>
-      <xdr:row>32</xdr:row>
-      <xdr:rowOff>125965</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>18</xdr:row>
+      <xdr:rowOff>92162</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>42823</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>125965</xdr:rowOff>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>167741</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="60" name="Liguster-Hecke_0_Text" descr="wep-app"/>
+        <xdr:cNvPr id="49" name="hecke_0" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="3597362"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>19</xdr:row>
+      <xdr:rowOff>85428</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>161007</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="50" name="hecke_1" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="3781128"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>20</xdr:row>
+      <xdr:rowOff>80609</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>156188</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="51" name="hecke_2" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="3966809"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>21</xdr:row>
+      <xdr:rowOff>73876</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>149455</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="52" name="hecke_3" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="4150576"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>67143</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>142722</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="53" name="hecke_4" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="4334343"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>62323</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>137902</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="54" name="hecke_5" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="4520023"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>55590</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>131169</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="55" name="hecke_6" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="4703790"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>48857</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>124436</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="56" name="hecke_7" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="4887557"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>41166</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>116745</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="57" name="hecke_8" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="5070366"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>27</xdr:row>
+      <xdr:rowOff>37304</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>112883</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="58" name="hecke_9" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="5257004"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>30571</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>106150</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="59" name="hecke_10" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="5440771"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>29</xdr:row>
+      <xdr:rowOff>22881</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>98460</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="60" name="hecke_11" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="5623581"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>118568</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>19019</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>384647</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>94598</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="61" name="hecke_12" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5376368" y="5810219"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>172167</xdr:colOff>
+      <xdr:row>31</xdr:row>
+      <xdr:rowOff>12285</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>438246</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>87864</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="62" name="hecke_13" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="5429967" y="5993985"/>
+          <a:ext cx="266079" cy="266079"/>
+        </a:xfrm>
+        <a:prstGeom prst="ellipse">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="A9D18E"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>461217</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>10572</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>103712</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>10572</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="63" name="hecke_14" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6052463" y="6298165"/>
-          <a:ext cx="981710" cy="190500"/>
+          <a:off x="5719017" y="4849272"/>
+          <a:ext cx="604520" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -19593,7 +19743,7 @@
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
             </a:rPr>
-            <a:t>Liguster-Hecke</a:t>
+            <a:t>Liguster</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -19603,24 +19753,167 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>158760</xdr:colOff>
-      <xdr:row>39</xdr:row>
-      <xdr:rowOff>29912</xdr:rowOff>
+      <xdr:colOff>192701</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>42612</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>700415</xdr:colOff>
-      <xdr:row>40</xdr:row>
-      <xdr:rowOff>29912</xdr:rowOff>
+      <xdr:colOff>666474</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>147862</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="61" name="Kompost_0_Text" descr="wep-app"/>
+        <xdr:cNvPr id="64" name="kompost_0" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="802301" y="7738812"/>
+          <a:ext cx="473773" cy="295750"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:solidFill>
+          <a:srgbClr val="D9C3A5"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="8B5A2B"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>310426</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>55054</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>310426</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>136376</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="65" name="kompost_1" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="920026" y="7751254"/>
+          <a:ext cx="0" cy="271822"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="31750">
+          <a:solidFill>
+            <a:srgbClr val="8B5A2B"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>429109</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>55054</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>429109</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>136376</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="66" name="kompost_2" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1038709" y="7751254"/>
+          <a:ext cx="0" cy="271822"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="31750">
+          <a:solidFill>
+            <a:srgbClr val="8B5A2B"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>547791</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>55054</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>547791</xdr:colOff>
+      <xdr:row>41</xdr:row>
+      <xdr:rowOff>136376</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="67" name="kompost_3" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1157391" y="7751254"/>
+          <a:ext cx="0" cy="271822"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="31750">
+          <a:solidFill>
+            <a:srgbClr val="8B5A2B"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>208972</xdr:colOff>
+      <xdr:row>39</xdr:row>
+      <xdr:rowOff>89544</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>750627</xdr:colOff>
+      <xdr:row>40</xdr:row>
+      <xdr:rowOff>89544</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="68" name="kompost_4" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="768360" y="7535612"/>
+          <a:off x="818572" y="7595244"/>
           <a:ext cx="541655" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -19653,27 +19946,240 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>44930</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>105875</xdr:rowOff>
+      <xdr:colOff>526735</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>82389</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>184630</xdr:colOff>
-      <xdr:row>23</xdr:row>
-      <xdr:rowOff>118575</xdr:rowOff>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>925853</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>100508</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="62" name="Blaufichte_entfernen_0_Hinweis" descr="wep-app"/>
+        <xdr:cNvPr id="69" name="entfernen_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="654530" y="4373075"/>
-          <a:ext cx="1358900" cy="203200"/>
+          <a:off x="1136335" y="4730589"/>
+          <a:ext cx="399118" cy="399119"/>
         </a:xfrm>
-        <a:prstGeom prst="roundRect">
+        <a:custGeom>
+          <a:avLst/>
+          <a:gdLst/>
+          <a:ahLst/>
+          <a:cxnLst/>
+          <a:rect l="l" t="t" r="r" b="b"/>
+          <a:pathLst>
+            <a:path w="399118" h="399119">
+              <a:moveTo>
+                <a:pt x="198123" y="0"/>
+              </a:moveTo>
+              <a:lnTo>
+                <a:pt x="227794" y="44028"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="275650" y="14357"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="284264" y="67956"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="340734" y="55513"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="328291" y="111983"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="381890" y="120597"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="352219" y="168453"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="399118" y="198124"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="352219" y="227795"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="381890" y="274693"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="328291" y="284265"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="340734" y="339777"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="284264" y="328292"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="275650" y="381891"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="227794" y="352220"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="198123" y="399119"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="168453" y="352220"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="121554" y="381891"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="112940" y="328292"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="56470" y="339777"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="67955" y="284265"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="15314" y="274693"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="44027" y="227795"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="0" y="198124"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="44027" y="168453"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="15314" y="120597"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="67955" y="111983"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="56470" y="55513"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="112940" y="67956"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="121554" y="14357"/>
+              </a:lnTo>
+              <a:lnTo>
+                <a:pt x="168453" y="44028"/>
+              </a:lnTo>
+              <a:close/>
+            </a:path>
+          </a:pathLst>
+        </a:custGeom>
+        <a:solidFill>
+          <a:srgbClr val="70AD47"/>
+        </a:solidFill>
+        <a:ln w="12700">
+          <a:solidFill>
+            <a:srgbClr val="548235"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>607133</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>161830</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>846412</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>21067</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="70" name="entfernen_1" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1216733" y="4810030"/>
+          <a:ext cx="239279" cy="240237"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>607133</xdr:colOff>
+      <xdr:row>24</xdr:row>
+      <xdr:rowOff>161830</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>846412</xdr:colOff>
+      <xdr:row>26</xdr:row>
+      <xdr:rowOff>21067</xdr:rowOff>
+    </xdr:to>
+    <xdr:cxnSp macro="">
+      <xdr:nvCxnSpPr>
+        <xdr:cNvPr id="71" name="entfernen_2" descr="wep-app"/>
+        <xdr:cNvCxnSpPr/>
+      </xdr:nvCxnSpPr>
+      <xdr:spPr>
+        <a:xfrm flipH="1">
+          <a:off x="1216733" y="4810030"/>
+          <a:ext cx="239279" cy="240237"/>
+        </a:xfrm>
+        <a:prstGeom prst="straightConnector1">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:ln w="25400">
+          <a:solidFill>
+            <a:srgbClr val="C00000"/>
+          </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:cxnSp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>13720</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>156155</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>217755</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>163778</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="72" name="entfernen_3" descr="wep-app"/>
+        <xdr:cNvSpPr/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="623320" y="4423355"/>
+          <a:ext cx="1423235" cy="198123"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
@@ -19683,6 +20189,40 @@
           <a:solidFill>
             <a:srgbClr val="C00000"/>
           </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>96032</xdr:colOff>
+      <xdr:row>22</xdr:row>
+      <xdr:rowOff>181997</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>235732</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>181997</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="73" name="entfernen_4" descr="wep-app"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="705632" y="4449197"/>
+          <a:ext cx="1358900" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
@@ -19707,25 +20247,25 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>724380</xdr:colOff>
+      <xdr:colOff>724858</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>118575</xdr:rowOff>
+      <xdr:rowOff>165692</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>2</xdr:col>
-      <xdr:colOff>724380</xdr:colOff>
+      <xdr:colOff>724858</xdr:colOff>
       <xdr:row>24</xdr:row>
-      <xdr:rowOff>80475</xdr:rowOff>
+      <xdr:rowOff>82389</xdr:rowOff>
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="63" name="Blaufichte_entfernen_0_Pfeil" descr="wep-app"/>
+        <xdr:cNvPr id="74" name="entfernen_5" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1333980" y="4576275"/>
-          <a:ext cx="0" cy="152400"/>
+          <a:off x="1334458" y="4623392"/>
+          <a:ext cx="0" cy="107197"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -19755,7 +20295,7 @@
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="64" name="Rückschnitt_nötig_0" descr="wep-app"/>
+        <xdr:cNvPr id="75" name="mangelhinweis_0" descr="wep-app"/>
         <xdr:cNvSpPr/>
       </xdr:nvSpPr>
       <xdr:spPr>
@@ -19763,7 +20303,7 @@
           <a:off x="1334458" y="6866877"/>
           <a:ext cx="1183955" cy="266079"/>
         </a:xfrm>
-        <a:prstGeom prst="roundRect">
+        <a:prstGeom prst="rect">
           <a:avLst/>
         </a:prstGeom>
         <a:solidFill>
@@ -19773,6 +20313,40 @@
           <a:solidFill>
             <a:srgbClr val="C00000"/>
           </a:solidFill>
+        </a:ln>
+      </xdr:spPr>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>781328</xdr:colOff>
+      <xdr:row>35</xdr:row>
+      <xdr:rowOff>176776</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>732433</xdr:colOff>
+      <xdr:row>36</xdr:row>
+      <xdr:rowOff>176776</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="76" name="mangelhinweis_1" descr="wep-app"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1390928" y="6920476"/>
+          <a:ext cx="1170305" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
         </a:ln>
       </xdr:spPr>
       <xdr:txBody>
@@ -19797,7 +20371,7 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>230747</xdr:colOff>
+      <xdr:colOff>231154</xdr:colOff>
       <xdr:row>37</xdr:row>
       <xdr:rowOff>8256</xdr:rowOff>
     </xdr:from>
@@ -19809,13 +20383,13 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="65" name="Rückschnitt_nötig_0_Pfeil" descr="wep-app"/>
+        <xdr:cNvPr id="77" name="mangelhinweis_2" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="2059547" y="7132956"/>
-          <a:ext cx="754616" cy="754209"/>
+          <a:off x="2059954" y="7132956"/>
+          <a:ext cx="754209" cy="754209"/>
         </a:xfrm>
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
@@ -19845,7 +20419,7 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="66" name="Pfeil_0" descr="wep-app"/>
+        <xdr:cNvPr id="78" name="Pfeil_0" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -19856,7 +20430,7 @@
         <a:prstGeom prst="straightConnector1">
           <a:avLst/>
         </a:prstGeom>
-        <a:ln w="12700">
+        <a:ln w="19050">
           <a:solidFill>
             <a:srgbClr val="C00000"/>
           </a:solidFill>
@@ -19881,7 +20455,7 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="67" name="Maß_0" descr="wep-app"/>
+        <xdr:cNvPr id="79" name="Maß_0" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -19916,7 +20490,7 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="68" name="Maß_0_Strich1" descr="wep-app"/>
+        <xdr:cNvPr id="80" name="Maß_0_Strich1" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -19951,7 +20525,7 @@
     </xdr:to>
     <xdr:cxnSp macro="">
       <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="69" name="Maß_0_Strich2" descr="wep-app"/>
+        <xdr:cNvPr id="81" name="Maß_0_Strich2" descr="wep-app"/>
         <xdr:cNvCxnSpPr/>
       </xdr:nvCxnSpPr>
       <xdr:spPr>
@@ -19974,24 +20548,24 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1483043</xdr:colOff>
+      <xdr:colOff>1104583</xdr:colOff>
       <xdr:row>6</xdr:row>
       <xdr:rowOff>74087</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1836103</xdr:colOff>
+      <xdr:colOff>1457643</xdr:colOff>
       <xdr:row>7</xdr:row>
       <xdr:rowOff>74087</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="70" name="Maß_0_Text" descr="wep-app"/>
+        <xdr:cNvPr id="82" name="Maß_0_Text" descr="wep-app"/>
         <xdr:cNvSpPr txBox="1"/>
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="3311843" y="1293287"/>
+          <a:off x="2933383" y="1293287"/>
           <a:ext cx="353060" cy="190500"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -20015,6 +20589,56 @@
               <a:latin typeface="+mn-lt"/>
             </a:rPr>
             <a:t>16 m</a:t>
+          </a:r>
+        </a:p>
+      </xdr:txBody>
+    </xdr:sp>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>454032</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>114309</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>995687</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>114309</xdr:rowOff>
+    </xdr:to>
+    <xdr:sp macro="" textlink="">
+      <xdr:nvSpPr>
+        <xdr:cNvPr id="83" name="Flieder_0_Text" descr="wep-app"/>
+        <xdr:cNvSpPr txBox="1"/>
+      </xdr:nvSpPr>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1063632" y="3048009"/>
+          <a:ext cx="541655" cy="190500"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </xdr:spPr>
+      <xdr:txBody>
+        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" lIns="12700" tIns="0" rIns="12700" bIns="0" rtlCol="0" anchor="ctr"/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr algn="ctr"/>
+          <a:r>
+            <a:rPr lang="de-DE" sz="900">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="+mn-lt"/>
+            </a:rPr>
+            <a:t>Flieder</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>

</xml_diff>